<commit_message>
File extended to 2070
</commit_message>
<xml_diff>
--- a/InputData/elec/BPHC/BAU Pumped Hydro Cap.xlsx
+++ b/InputData/elec/BPHC/BAU Pumped Hydro Cap.xlsx
@@ -1,31 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10119"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ssy02/Desktop/Postdoc Projects/eps-indonesia-cpl/InputData/elec/BPHC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B32FD36-1CE3-FE45-BD79-8CF2B8FE7FA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF2A7192-1C32-DF46-A18D-A3A60C60E5E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34200" windowHeight="21380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="21360" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
     <sheet name="BPHC" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlchart.v1.0" hidden="1">BPHC!$A$1</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">BPHC!$A$2</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">BPHC!$B$1:$AL$1</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">BPHC!$B$2:$AL$2</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">BPHC!$A$1</definedName>
-    <definedName name="_xlchart.v1.5" hidden="1">BPHC!$A$2</definedName>
-    <definedName name="_xlchart.v1.6" hidden="1">BPHC!$B$1:$AL$1</definedName>
-    <definedName name="_xlchart.v1.7" hidden="1">BPHC!$B$2:$AL$2</definedName>
-  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -86,7 +76,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -117,6 +107,13 @@
       <color theme="10"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -153,7 +150,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -172,6 +169,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1441,14 +1439,14 @@
   <sheetPr>
     <tabColor rgb="FF1F497D"/>
   </sheetPr>
-  <dimension ref="A1:AL1000"/>
+  <dimension ref="A1:BG1000"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="26.6640625" customWidth="1"/>
     <col min="2" max="38" width="7.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:59" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
         <v>4</v>
       </c>
@@ -1563,8 +1561,89 @@
       <c r="AL1" s="5">
         <v>2050</v>
       </c>
+      <c r="AM1" s="10">
+        <f>AL1+1</f>
+        <v>2051</v>
+      </c>
+      <c r="AN1" s="10">
+        <f t="shared" ref="AN1:BG1" si="0">AM1+1</f>
+        <v>2052</v>
+      </c>
+      <c r="AO1" s="10">
+        <f t="shared" si="0"/>
+        <v>2053</v>
+      </c>
+      <c r="AP1" s="10">
+        <f t="shared" si="0"/>
+        <v>2054</v>
+      </c>
+      <c r="AQ1" s="10">
+        <f t="shared" si="0"/>
+        <v>2055</v>
+      </c>
+      <c r="AR1" s="10">
+        <f t="shared" si="0"/>
+        <v>2056</v>
+      </c>
+      <c r="AS1" s="10">
+        <f t="shared" si="0"/>
+        <v>2057</v>
+      </c>
+      <c r="AT1" s="10">
+        <f t="shared" si="0"/>
+        <v>2058</v>
+      </c>
+      <c r="AU1" s="10">
+        <f t="shared" si="0"/>
+        <v>2059</v>
+      </c>
+      <c r="AV1" s="10">
+        <f t="shared" si="0"/>
+        <v>2060</v>
+      </c>
+      <c r="AW1" s="10">
+        <f t="shared" si="0"/>
+        <v>2061</v>
+      </c>
+      <c r="AX1" s="10">
+        <f t="shared" si="0"/>
+        <v>2062</v>
+      </c>
+      <c r="AY1" s="10">
+        <f t="shared" si="0"/>
+        <v>2063</v>
+      </c>
+      <c r="AZ1" s="10">
+        <f t="shared" si="0"/>
+        <v>2064</v>
+      </c>
+      <c r="BA1" s="10">
+        <f t="shared" si="0"/>
+        <v>2065</v>
+      </c>
+      <c r="BB1" s="10">
+        <f t="shared" si="0"/>
+        <v>2066</v>
+      </c>
+      <c r="BC1" s="10">
+        <f t="shared" si="0"/>
+        <v>2067</v>
+      </c>
+      <c r="BD1" s="10">
+        <f t="shared" si="0"/>
+        <v>2068</v>
+      </c>
+      <c r="BE1" s="10">
+        <f t="shared" si="0"/>
+        <v>2069</v>
+      </c>
+      <c r="BF1" s="10">
+        <f t="shared" si="0"/>
+        <v>2070</v>
+      </c>
+      <c r="BG1" s="10"/>
     </row>
-    <row r="2" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:59" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>5</v>
       </c>
@@ -1603,15 +1682,15 @@
         <v>1983</v>
       </c>
       <c r="M2" s="7">
-        <f t="shared" ref="M2:AL2" si="0">L2</f>
+        <f t="shared" ref="M2:AL2" si="1">L2</f>
         <v>1983</v>
       </c>
       <c r="N2" s="7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1983</v>
       </c>
       <c r="O2" s="7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1983</v>
       </c>
       <c r="P2" s="7">
@@ -1619,108 +1698,188 @@
         <v>2983</v>
       </c>
       <c r="Q2" s="7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2983</v>
       </c>
       <c r="R2" s="7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2983</v>
       </c>
       <c r="S2" s="7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2983</v>
       </c>
       <c r="T2" s="7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2983</v>
       </c>
       <c r="U2" s="7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2983</v>
       </c>
       <c r="V2" s="7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2983</v>
       </c>
       <c r="W2" s="7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2983</v>
       </c>
       <c r="X2" s="7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2983</v>
       </c>
       <c r="Y2" s="7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2983</v>
       </c>
       <c r="Z2" s="7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2983</v>
       </c>
       <c r="AA2" s="7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2983</v>
       </c>
       <c r="AB2" s="7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2983</v>
       </c>
       <c r="AC2" s="7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2983</v>
       </c>
       <c r="AD2" s="7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2983</v>
       </c>
       <c r="AE2" s="7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2983</v>
       </c>
       <c r="AF2" s="7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2983</v>
       </c>
       <c r="AG2" s="7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2983</v>
       </c>
       <c r="AH2" s="7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2983</v>
       </c>
       <c r="AI2" s="7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2983</v>
       </c>
       <c r="AJ2" s="7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2983</v>
       </c>
       <c r="AK2" s="7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2983</v>
       </c>
       <c r="AL2" s="7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
+        <v>2983</v>
+      </c>
+      <c r="AM2" s="7">
+        <f t="shared" ref="AM2" si="2">AL2</f>
+        <v>2983</v>
+      </c>
+      <c r="AN2" s="7">
+        <f t="shared" ref="AN2" si="3">AM2</f>
+        <v>2983</v>
+      </c>
+      <c r="AO2" s="7">
+        <f t="shared" ref="AO2" si="4">AN2</f>
+        <v>2983</v>
+      </c>
+      <c r="AP2" s="7">
+        <f t="shared" ref="AP2" si="5">AO2</f>
+        <v>2983</v>
+      </c>
+      <c r="AQ2" s="7">
+        <f t="shared" ref="AQ2" si="6">AP2</f>
+        <v>2983</v>
+      </c>
+      <c r="AR2" s="7">
+        <f t="shared" ref="AR2" si="7">AQ2</f>
+        <v>2983</v>
+      </c>
+      <c r="AS2" s="7">
+        <f t="shared" ref="AS2" si="8">AR2</f>
+        <v>2983</v>
+      </c>
+      <c r="AT2" s="7">
+        <f t="shared" ref="AT2" si="9">AS2</f>
+        <v>2983</v>
+      </c>
+      <c r="AU2" s="7">
+        <f t="shared" ref="AU2" si="10">AT2</f>
+        <v>2983</v>
+      </c>
+      <c r="AV2" s="7">
+        <f t="shared" ref="AV2" si="11">AU2</f>
+        <v>2983</v>
+      </c>
+      <c r="AW2" s="7">
+        <f t="shared" ref="AW2" si="12">AV2</f>
+        <v>2983</v>
+      </c>
+      <c r="AX2" s="7">
+        <f t="shared" ref="AX2" si="13">AW2</f>
+        <v>2983</v>
+      </c>
+      <c r="AY2" s="7">
+        <f t="shared" ref="AY2" si="14">AX2</f>
+        <v>2983</v>
+      </c>
+      <c r="AZ2" s="7">
+        <f t="shared" ref="AZ2" si="15">AY2</f>
+        <v>2983</v>
+      </c>
+      <c r="BA2" s="7">
+        <f t="shared" ref="BA2" si="16">AZ2</f>
+        <v>2983</v>
+      </c>
+      <c r="BB2" s="7">
+        <f t="shared" ref="BB2" si="17">BA2</f>
+        <v>2983</v>
+      </c>
+      <c r="BC2" s="7">
+        <f t="shared" ref="BC2" si="18">BB2</f>
+        <v>2983</v>
+      </c>
+      <c r="BD2" s="7">
+        <f t="shared" ref="BD2" si="19">BC2</f>
+        <v>2983</v>
+      </c>
+      <c r="BE2" s="7">
+        <f t="shared" ref="BE2" si="20">BD2</f>
+        <v>2983</v>
+      </c>
+      <c r="BF2" s="7">
+        <f t="shared" ref="BF2" si="21">BE2</f>
         <v>2983</v>
       </c>
     </row>
-    <row r="3" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="4" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="5" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="6" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="7" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="8" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="9" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="10" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="11" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="12" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="13" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="14" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="15" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="16" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="3" spans="1:59" ht="14.25" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="4" spans="1:59" ht="14.25" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="5" spans="1:59" ht="14.25" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="6" spans="1:59" ht="14.25" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="7" spans="1:59" ht="14.25" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="8" spans="1:59" ht="14.25" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="9" spans="1:59" ht="14.25" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="10" spans="1:59" ht="14.25" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="11" spans="1:59" ht="14.25" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="12" spans="1:59" ht="14.25" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="13" spans="1:59" ht="14.25" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="14" spans="1:59" ht="14.25" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="15" spans="1:59" ht="14.25" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="16" spans="1:59" ht="14.25" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="17" ht="14.25" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="18" ht="14.25" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="19" ht="14.25" customHeight="1" x14ac:dyDescent="0.15"/>
@@ -2708,5 +2867,8 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
+  <ignoredErrors>
+    <ignoredError sqref="P2" formula="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>